<commit_message>
nastavak Senj zadataka, procitaj bilj
</commit_message>
<xml_diff>
--- a/HE_Senj/HE Senj - rashlada - specifikacija opreme_FŠ -- rv.xlsx
+++ b/HE_Senj/HE Senj - rashlada - specifikacija opreme_FŠ -- rv.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\odojak\Brodotehna\Projekti\HE_Senj\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9464A7D4-4823-4FA2-BF06-57D62831D833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{EBE008FF-735A-4426-A2DE-3EF07B854623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-4155" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{324E8A42-1211-42FF-BECF-D2BB17870C58}"/>
+    <workbookView xWindow="-38535" yWindow="-4170" windowWidth="38670" windowHeight="21150" activeTab="1" xr2:uid="{324E8A42-1211-42FF-BECF-D2BB17870C58}"/>
   </bookViews>
   <sheets>
     <sheet name="Zadaci" sheetId="1" r:id="rId1"/>
     <sheet name="Specifikacija_opreme_-_HEP-v2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Specifikacija_opreme_-_HEP-v2'!$B$1:$F$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Specifikacija_opreme_-_HEP-v2'!$B$1:$F$115</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
     <author/>
   </authors>
   <commentList>
-    <comment ref="D113" authorId="0" shapeId="1025" xr:uid="{C8BB19DC-EE89-4F88-A3A7-D88407000A4D}">
+    <comment ref="D112" authorId="0" shapeId="1025" xr:uid="{C8BB19DC-EE89-4F88-A3A7-D88407000A4D}">
       <text>
         <r>
           <rPr>
@@ -66,14 +67,14 @@
               <from>
                 <xdr:col>7</xdr:col>
                 <xdr:colOff>563880</xdr:colOff>
-                <xdr:row>154</xdr:row>
-                <xdr:rowOff>99060</xdr:rowOff>
+                <xdr:row>151</xdr:row>
+                <xdr:rowOff>144780</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>8</xdr:col>
                 <xdr:colOff>533400</xdr:colOff>
-                <xdr:row>159</xdr:row>
-                <xdr:rowOff>99060</xdr:rowOff>
+                <xdr:row>156</xdr:row>
+                <xdr:rowOff>144780</xdr:rowOff>
               </to>
             </anchor>
           </commentPr>
@@ -85,7 +86,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="710" uniqueCount="336">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="704" uniqueCount="333">
   <si>
     <t>Br zadatka</t>
   </si>
@@ -556,16 +557,9 @@
     <t>Končar</t>
   </si>
   <si>
-    <t>-H4, -H5, -H6, -H7, -H102, -H202, -H302, -H402, -H502, -H602, -H701, -H702, -H703, H801, -H802</t>
-  </si>
-  <si>
     <t>Svjetleće tijelo, leća: CRVENA, prednji okvir: sivi; 35×35mm, podnožje za sijalicu sa vijčanim priključkom</t>
   </si>
   <si>
-    <t>nije upisan part u EPLANu; 
-ne postoje -H6, -H7, -H701, -H702, -H703, H801, -H802</t>
-  </si>
-  <si>
     <t>-H1, -H2, -H3, -H401, -H501, -H601</t>
   </si>
   <si>
@@ -576,9 +570,6 @@
   </si>
   <si>
     <t>nije upisan part u EPLANu</t>
-  </si>
-  <si>
-    <t>-H8, -H101, -H201, -H301, -H404, -H504, -H604</t>
   </si>
   <si>
     <t>Svjetleće tijelo, leća: PROZIRNA, prednji okvir: sivi; 35×35mm, podnožje za sijalicu sa vijčanim priključkom</t>
@@ -600,9 +591,6 @@
     <t>704.202.408</t>
   </si>
   <si>
-    <t>-S110, -S101, -S201, -S301</t>
-  </si>
-  <si>
     <t>Svjetleće tipkalo, leća: CRVENA, prednji okvir: crni; 35×35mm, podnožje za sijalicu sa vijčanim priključkom</t>
   </si>
   <si>
@@ -676,9 +664,6 @@
     <t>LAD9R1V</t>
   </si>
   <si>
-    <t>koristi se stavka iznad</t>
-  </si>
-  <si>
     <t>-FU1</t>
   </si>
   <si>
@@ -857,20 +842,6 @@
   </si>
   <si>
     <t>IME</t>
-  </si>
-  <si>
-    <t>ne postoji -P101 u EPLANu nego samo -V1</t>
-  </si>
-  <si>
-    <t>-V1</t>
-  </si>
-  <si>
-    <t>voltmetar 0 - 400 V
-Part number: IME.AN25DDC400</t>
-  </si>
-  <si>
-    <t>dodano; 
-nema nar. br. u summarized parts listi</t>
   </si>
   <si>
     <t>-P201, -P202</t>
@@ -959,9 +930,6 @@
   </si>
   <si>
     <t>Distributor za 24 VDC- 1-polni distribucijski blok, za bakrene vodiče, priključne stezaljke: ulazne 2 x 25mm², izlazne 6 x (1.5 – 10mm²), montaža na DIN nosač ili na montažnu ploču, nazivna struja IEC: 100A, 54x29x50mm (VxŠxD)</t>
-  </si>
-  <si>
-    <t>IKB01025N</t>
   </si>
   <si>
     <t>u summarized parts listi su još i -X505, -X550, -X551; 
@@ -1120,12 +1088,6 @@
     <t>PK: Dodati kataloški broj u jednu od dioda</t>
   </si>
   <si>
-    <t>PK: Ovo je -P101</t>
-  </si>
-  <si>
-    <t>PK: Ovo ne treba biti u shemama</t>
-  </si>
-  <si>
     <t>PK: Ja moram pronaći alternativu</t>
   </si>
   <si>
@@ -1153,19 +1115,144 @@
     <t>PK: Stranica shema 121 na releje K102.1 i K103.1 te str 74 na releje -2K12 i -2K13</t>
   </si>
   <si>
-    <t>PK: Dodati "-" kao sufiks. Ja moram provjeriti naručene količine</t>
+    <t>IKB01025N-</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PK: </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Dodati "-" kao sufiks.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Ja moram provjeriti naručene količine</t>
+    </r>
+  </si>
+  <si>
+    <t>nije upisan part u EPLANu; 
+ne postoje -H6, -H7, -H701, -H702, -H703, -H801, -H802</t>
+  </si>
+  <si>
+    <t>EAO.10-2512.1149</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">-H8, </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-H101, -H201, -H301,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> -H404, -H504, -H604</t>
+    </r>
+  </si>
+  <si>
+    <t>EAO.704.911.5-1</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">-S110, </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-S101, -S201, -S301</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">-H4, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-H5, -H6, -H7,</t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> -H102, -H202, -H302, -H402, -H502, -H602, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-H701, -H702, -H703, H801, -H802</t>
+    </r>
+  </si>
+  <si>
+    <t>EAO.704.229.500</t>
+  </si>
+  <si>
+    <t>704.209.700</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1211,8 +1298,43 @@
       <family val="2"/>
       <charset val="238"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1251,12 +1373,28 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="12">
     <border>
       <start/>
       <end/>
@@ -1370,32 +1508,78 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <start style="thin">
+        <color rgb="FFB2B2B2"/>
+      </start>
+      <end style="thin">
+        <color rgb="FFB2B2B2"/>
+      </end>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <start style="thin">
+        <color indexed="64"/>
+      </start>
+      <end style="thin">
+        <color indexed="64"/>
+      </end>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <start/>
+      <end style="thin">
+        <color rgb="FF000000"/>
+      </end>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="8">
+  <cellStyleXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" applyBorder="0" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1428,18 +1612,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1454,16 +1632,97 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="5" xfId="10" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="9" borderId="5" xfId="10" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="5" xfId="10" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="7" borderId="10" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" xfId="8" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="10" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="10" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="8" borderId="10" xfId="9" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="10" xfId="9" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="8">
+  <cellStyles count="11">
+    <cellStyle name="20% - Accent2" xfId="10" builtinId="34"/>
     <cellStyle name="40% - Accent1 3 2" xfId="1" xr:uid="{222F9BCB-D27A-412B-A74C-613EC62AF50A}"/>
     <cellStyle name="cf1" xfId="2" xr:uid="{54248B18-6E67-40DC-A6F6-C25F5815B94F}"/>
     <cellStyle name="cf2" xfId="3" xr:uid="{054CFDE7-787D-4501-BDB9-B0A0F5413F8A}"/>
     <cellStyle name="cf3" xfId="4" xr:uid="{DB55E99D-B714-474C-B9EB-450368BA8106}"/>
     <cellStyle name="ColStyle3" xfId="5" xr:uid="{F2DAC5EA-D14E-477E-B90F-4F365988442E}"/>
+    <cellStyle name="Good" xfId="8" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
     <cellStyle name="Normal 2" xfId="6" xr:uid="{E19DF288-7D14-4C51-AC68-B5DE90415F70}"/>
     <cellStyle name="Normal 2 5" xfId="7" xr:uid="{CE5137AD-0C1F-4639-9579-8CD0BF4D72B1}"/>
+    <cellStyle name="Note" xfId="9" builtinId="10"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -1500,21 +1759,21 @@
         <xdr:from>
           <xdr:col>7</xdr:col>
           <xdr:colOff>563880</xdr:colOff>
-          <xdr:row>154</xdr:row>
-          <xdr:rowOff>99060</xdr:rowOff>
+          <xdr:row>151</xdr:row>
+          <xdr:rowOff>144780</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>8</xdr:col>
           <xdr:colOff>533400</xdr:colOff>
-          <xdr:row>159</xdr:row>
-          <xdr:rowOff>99060</xdr:rowOff>
+          <xdr:row>156</xdr:row>
+          <xdr:rowOff>144780</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="1025" name="Comment 1" hidden="1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5A3C7C2B-5065-0F8B-6F0E-9ADC013BFD27}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F5258D2A-04CB-1B71-4553-2CE847E28268}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1524,7 +1783,7 @@
           </xdr:nvSpPr>
           <xdr:spPr bwMode="auto">
             <a:xfrm>
-              <a:off x="13296900" y="68961000"/>
+              <a:off x="13296900" y="68778120"/>
               <a:ext cx="1828800" cy="914400"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -1957,7 +2216,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:xdr="http://purl.oclc.org/ooxml/drawingml/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0791F9D3-C3E8-4198-906E-F1EBBAF01A10}">
-  <dimension ref="A1:K126"/>
+  <dimension ref="A1:K125"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="39" style="1" customWidth="1"/>
@@ -1970,7 +2229,7 @@
     <col min="8" max="8" width="27.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="46.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="48.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="23.4" customHeight="1" thickBot="1">
@@ -2005,7 +2264,7 @@
         <v>13</v>
       </c>
       <c r="K1" s="20" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="30.6" customHeight="1">
@@ -2593,7 +2852,7 @@
         <v>-2</v>
       </c>
       <c r="K22" s="19" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="30.6" customHeight="1">
@@ -2686,8 +2945,8 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K25" s="19" t="s">
-        <v>310</v>
+      <c r="K25" s="28" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="94.2" customHeight="1">
@@ -2932,15 +3191,15 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="88.95" customHeight="1">
+    <row r="34" spans="1:11" ht="121.8" customHeight="1">
       <c r="A34" s="21" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>56</v>
@@ -2961,8 +3220,8 @@
       <c r="J34" s="11">
         <v>1</v>
       </c>
-      <c r="K34" t="s">
-        <v>316</v>
+      <c r="K34" s="29" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="57.6">
@@ -3267,7 +3526,7 @@
         <v>-2</v>
       </c>
       <c r="K44" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="43.2">
@@ -3330,7 +3589,7 @@
         <v>19</v>
       </c>
       <c r="K46" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="57.6">
@@ -3393,7 +3652,7 @@
         <v>-3</v>
       </c>
       <c r="K48" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="72">
@@ -3429,7 +3688,7 @@
         <v>-7</v>
       </c>
       <c r="K49" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="72">
@@ -3465,7 +3724,7 @@
         <v>-17</v>
       </c>
       <c r="K50" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="43.2">
@@ -3550,8 +3809,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K53" t="s">
-        <v>319</v>
+      <c r="K53" s="29" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="54" spans="1:11" ht="28.8">
@@ -3802,19 +4061,19 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K62" s="19" t="s">
-        <v>320</v>
+      <c r="K62" s="31" t="s">
+        <v>310</v>
       </c>
     </row>
     <row r="63" spans="1:11" ht="26.4" customHeight="1">
-      <c r="A63" s="9"/>
-      <c r="B63" s="9" t="s">
+      <c r="A63" s="36"/>
+      <c r="B63" s="36" t="s">
         <v>136</v>
       </c>
-      <c r="C63" s="10" t="s">
+      <c r="C63" s="37" t="s">
         <v>137</v>
       </c>
-      <c r="D63" s="11" t="s">
+      <c r="D63" s="38" t="s">
         <v>138</v>
       </c>
       <c r="E63" s="11">
@@ -3834,14 +4093,14 @@
       </c>
     </row>
     <row r="64" spans="1:11" ht="26.4" customHeight="1">
-      <c r="A64" s="9"/>
-      <c r="B64" s="9" t="s">
+      <c r="A64" s="36"/>
+      <c r="B64" s="36" t="s">
         <v>139</v>
       </c>
-      <c r="C64" s="10" t="s">
+      <c r="C64" s="37" t="s">
         <v>140</v>
       </c>
-      <c r="D64" s="11" t="s">
+      <c r="D64" s="38" t="s">
         <v>138</v>
       </c>
       <c r="E64" s="11">
@@ -3861,14 +4120,14 @@
       </c>
     </row>
     <row r="65" spans="1:11" ht="26.4" customHeight="1">
-      <c r="A65" s="9"/>
-      <c r="B65" s="9" t="s">
+      <c r="A65" s="36"/>
+      <c r="B65" s="36" t="s">
         <v>141</v>
       </c>
-      <c r="C65" s="10" t="s">
+      <c r="C65" s="37" t="s">
         <v>142</v>
       </c>
-      <c r="D65" s="11" t="s">
+      <c r="D65" s="38" t="s">
         <v>138</v>
       </c>
       <c r="E65" s="11">
@@ -3888,14 +4147,14 @@
       </c>
     </row>
     <row r="66" spans="1:11" ht="26.4" customHeight="1">
-      <c r="A66" s="9"/>
-      <c r="B66" s="9" t="s">
+      <c r="A66" s="36"/>
+      <c r="B66" s="36" t="s">
         <v>143</v>
       </c>
-      <c r="C66" s="10" t="s">
+      <c r="C66" s="37" t="s">
         <v>144</v>
       </c>
-      <c r="D66" s="11" t="s">
+      <c r="D66" s="38" t="s">
         <v>138</v>
       </c>
       <c r="E66" s="11">
@@ -3915,16 +4174,16 @@
       </c>
     </row>
     <row r="67" spans="1:11" ht="44.4" customHeight="1">
-      <c r="A67" s="9" t="s">
+      <c r="A67" s="40" t="s">
         <v>145</v>
       </c>
-      <c r="B67" s="9" t="s">
+      <c r="B67" s="40" t="s">
         <v>146</v>
       </c>
-      <c r="C67" s="10" t="s">
+      <c r="C67" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="D67" s="11" t="s">
+      <c r="D67" s="17" t="s">
         <v>148</v>
       </c>
       <c r="E67" s="11">
@@ -3944,24 +4203,24 @@
         <f t="shared" ref="J67:J98" si="2">IF(ISBLANK(I67),"",E67-I67)</f>
         <v>-5</v>
       </c>
-      <c r="K67" t="s">
-        <v>321</v>
+      <c r="K67" s="31" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="68" spans="1:11" ht="44.4" customHeight="1">
-      <c r="A68" s="9" t="s">
+      <c r="A68" s="54" t="s">
+        <v>330</v>
+      </c>
+      <c r="B68" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B68" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="C68" s="14" t="s">
-        <v>309</v>
-      </c>
-      <c r="D68" s="11" t="s">
+      <c r="C68" s="43" t="s">
+        <v>299</v>
+      </c>
+      <c r="D68" s="44" t="s">
         <v>138</v>
       </c>
-      <c r="E68" s="11">
+      <c r="E68" s="39">
         <v>15</v>
       </c>
       <c r="F68" s="11" t="s">
@@ -3971,41 +4230,41 @@
         <v>17</v>
       </c>
       <c r="H68" s="15" t="s">
-        <v>151</v>
+        <v>325</v>
       </c>
       <c r="I68" s="11"/>
       <c r="J68" s="7" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K68" s="19" t="s">
-        <v>322</v>
+      <c r="K68" s="30" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="69" spans="1:11" ht="44.4" customHeight="1">
-      <c r="A69" s="9" t="s">
+      <c r="A69" s="51" t="s">
+        <v>150</v>
+      </c>
+      <c r="B69" s="51" t="s">
+        <v>151</v>
+      </c>
+      <c r="C69" s="52" t="s">
         <v>152</v>
       </c>
-      <c r="B69" s="9" t="s">
+      <c r="D69" s="53" t="s">
+        <v>138</v>
+      </c>
+      <c r="E69" s="39">
+        <v>6</v>
+      </c>
+      <c r="F69" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G69" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H69" s="15" t="s">
         <v>153</v>
-      </c>
-      <c r="C69" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="D69" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="E69" s="11">
-        <v>6</v>
-      </c>
-      <c r="F69" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G69" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="H69" s="15" t="s">
-        <v>155</v>
       </c>
       <c r="I69" s="11"/>
       <c r="J69" s="7" t="str">
@@ -4014,29 +4273,29 @@
       </c>
     </row>
     <row r="70" spans="1:11" ht="44.4" customHeight="1">
-      <c r="A70" s="9" t="s">
+      <c r="A70" s="55" t="s">
+        <v>327</v>
+      </c>
+      <c r="B70" s="45" t="s">
+        <v>154</v>
+      </c>
+      <c r="C70" s="46" t="s">
+        <v>155</v>
+      </c>
+      <c r="D70" s="47" t="s">
+        <v>138</v>
+      </c>
+      <c r="E70" s="39">
+        <v>6</v>
+      </c>
+      <c r="F70" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G70" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H70" s="15" t="s">
         <v>156</v>
-      </c>
-      <c r="B70" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="C70" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="D70" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="E70" s="11">
-        <v>6</v>
-      </c>
-      <c r="F70" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G70" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="H70" s="15" t="s">
-        <v>159</v>
       </c>
       <c r="I70" s="11"/>
       <c r="J70" s="7" t="str">
@@ -4045,19 +4304,19 @@
       </c>
     </row>
     <row r="71" spans="1:11" ht="44.4" customHeight="1">
-      <c r="A71" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="B71" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="C71" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="D71" s="11" t="s">
+      <c r="A71" s="56" t="s">
+        <v>157</v>
+      </c>
+      <c r="B71" s="56" t="s">
+        <v>158</v>
+      </c>
+      <c r="C71" s="57" t="s">
+        <v>159</v>
+      </c>
+      <c r="D71" s="58" t="s">
         <v>138</v>
       </c>
-      <c r="E71" s="11">
+      <c r="E71" s="39">
         <v>3</v>
       </c>
       <c r="F71" s="11" t="s">
@@ -4067,7 +4326,7 @@
         <v>17</v>
       </c>
       <c r="H71" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="I71" s="11"/>
       <c r="J71" s="7" t="str">
@@ -4076,16 +4335,16 @@
       </c>
     </row>
     <row r="72" spans="1:11" ht="44.4" customHeight="1">
-      <c r="A72" s="9" t="s">
-        <v>163</v>
-      </c>
-      <c r="B72" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="C72" s="14" t="s">
-        <v>165</v>
-      </c>
-      <c r="D72" s="11" t="s">
+      <c r="A72" s="54" t="s">
+        <v>329</v>
+      </c>
+      <c r="B72" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="C72" s="43" t="s">
+        <v>161</v>
+      </c>
+      <c r="D72" s="44" t="s">
         <v>138</v>
       </c>
       <c r="E72" s="11">
@@ -4098,7 +4357,7 @@
         <v>17</v>
       </c>
       <c r="H72" s="9" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="I72" s="11">
         <v>4</v>
@@ -4109,16 +4368,16 @@
       </c>
     </row>
     <row r="73" spans="1:11" ht="44.4" customHeight="1">
-      <c r="A73" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="B73" s="9" t="s">
-        <v>168</v>
-      </c>
-      <c r="C73" s="14" t="s">
-        <v>169</v>
-      </c>
-      <c r="D73" s="11" t="s">
+      <c r="A73" s="51" t="s">
+        <v>163</v>
+      </c>
+      <c r="B73" s="51" t="s">
+        <v>164</v>
+      </c>
+      <c r="C73" s="52" t="s">
+        <v>165</v>
+      </c>
+      <c r="D73" s="53" t="s">
         <v>138</v>
       </c>
       <c r="E73" s="11">
@@ -4131,7 +4390,7 @@
         <v>17</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="I73" s="11">
         <v>3</v>
@@ -4142,16 +4401,16 @@
       </c>
     </row>
     <row r="74" spans="1:11" ht="44.4" customHeight="1">
-      <c r="A74" s="9" t="s">
-        <v>171</v>
-      </c>
-      <c r="B74" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="C74" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="D74" s="11" t="s">
+      <c r="A74" s="59" t="s">
+        <v>167</v>
+      </c>
+      <c r="B74" s="59" t="s">
+        <v>168</v>
+      </c>
+      <c r="C74" s="60" t="s">
+        <v>169</v>
+      </c>
+      <c r="D74" s="61" t="s">
         <v>138</v>
       </c>
       <c r="E74" s="11">
@@ -4164,7 +4423,7 @@
         <v>17</v>
       </c>
       <c r="H74" s="9" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="I74" s="11">
         <v>3</v>
@@ -4174,20 +4433,20 @@
         <v>0</v>
       </c>
       <c r="K74" s="19" t="s">
-        <v>323</v>
+        <v>313</v>
       </c>
     </row>
     <row r="75" spans="1:11" ht="43.2">
-      <c r="A75" s="9" t="s">
-        <v>171</v>
-      </c>
-      <c r="B75" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="C75" s="14">
-        <v>704209700</v>
-      </c>
-      <c r="D75" s="11" t="s">
+      <c r="A75" s="59" t="s">
+        <v>167</v>
+      </c>
+      <c r="B75" s="59" t="s">
+        <v>170</v>
+      </c>
+      <c r="C75" s="60" t="s">
+        <v>332</v>
+      </c>
+      <c r="D75" s="61" t="s">
         <v>138</v>
       </c>
       <c r="E75" s="11">
@@ -4200,7 +4459,7 @@
         <v>17</v>
       </c>
       <c r="H75" s="18" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
       <c r="I75" s="11"/>
       <c r="J75" s="7" t="str">
@@ -4209,16 +4468,16 @@
       </c>
     </row>
     <row r="76" spans="1:11" ht="28.8">
-      <c r="A76" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="B76" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="C76" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="D76" s="11" t="s">
+      <c r="A76" s="48" t="s">
+        <v>171</v>
+      </c>
+      <c r="B76" s="48" t="s">
+        <v>172</v>
+      </c>
+      <c r="C76" s="49" t="s">
+        <v>173</v>
+      </c>
+      <c r="D76" s="50" t="s">
         <v>138</v>
       </c>
       <c r="E76" s="11">
@@ -4240,16 +4499,16 @@
       </c>
     </row>
     <row r="77" spans="1:11">
-      <c r="A77" s="9" t="s">
+      <c r="A77" s="48" t="s">
+        <v>171</v>
+      </c>
+      <c r="B77" s="50" t="s">
+        <v>174</v>
+      </c>
+      <c r="C77" s="49" t="s">
         <v>175</v>
       </c>
-      <c r="B77" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="C77" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="D77" s="11" t="s">
+      <c r="D77" s="50" t="s">
         <v>138</v>
       </c>
       <c r="E77" s="11">
@@ -4272,13 +4531,13 @@
     </row>
     <row r="78" spans="1:11" ht="43.2">
       <c r="A78" s="9" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B78" s="9" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C78" s="10" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D78" s="11" t="s">
         <v>56</v>
@@ -4303,13 +4562,13 @@
     </row>
     <row r="79" spans="1:11" ht="28.8">
       <c r="A79" s="16" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B79" s="9" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C79" s="10" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D79" s="11" t="s">
         <v>51</v>
@@ -4331,19 +4590,19 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K79" s="1" t="s">
-        <v>324</v>
+      <c r="K79" s="32" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="80" spans="1:11" ht="28.8">
       <c r="A80" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="B80" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="C80" s="10" t="s">
         <v>183</v>
-      </c>
-      <c r="B80" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="C80" s="10" t="s">
-        <v>187</v>
       </c>
       <c r="D80" s="11" t="s">
         <v>51</v>
@@ -4357,30 +4616,28 @@
       <c r="G80" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H80" s="9" t="s">
-        <v>188</v>
-      </c>
+      <c r="H80" s="9"/>
       <c r="I80" s="11"/>
       <c r="J80" s="7" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K80" s="19" t="s">
-        <v>325</v>
+      <c r="K80" s="28" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="81" spans="1:11" ht="28.8">
       <c r="A81" s="9" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="B81" s="9" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C81" s="10">
         <v>943405</v>
       </c>
       <c r="D81" s="11" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="E81" s="11">
         <v>1</v>
@@ -4392,7 +4649,7 @@
         <v>17</v>
       </c>
       <c r="H81" s="9" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="I81" s="11">
         <v>1</v>
@@ -4404,16 +4661,16 @@
     </row>
     <row r="82" spans="1:11" ht="28.8">
       <c r="A82" s="9" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B82" s="9" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="C82" s="10">
         <v>93444012</v>
       </c>
       <c r="D82" s="11" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="E82" s="11">
         <v>1</v>
@@ -4435,16 +4692,16 @@
     </row>
     <row r="83" spans="1:11">
       <c r="A83" s="9" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B83" s="9" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C83" s="10">
         <v>13094006</v>
       </c>
       <c r="D83" s="11" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="E83" s="11">
         <v>1</v>
@@ -4466,16 +4723,16 @@
     </row>
     <row r="84" spans="1:11">
       <c r="A84" s="9" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B84" s="9" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="C84" s="10">
         <v>22944016</v>
       </c>
       <c r="D84" s="11" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="E84" s="11">
         <v>1</v>
@@ -4497,16 +4754,16 @@
     </row>
     <row r="85" spans="1:11">
       <c r="A85" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="B85" s="9" t="s">
         <v>192</v>
-      </c>
-      <c r="B85" s="9" t="s">
-        <v>197</v>
       </c>
       <c r="C85" s="10">
         <v>13994006</v>
       </c>
       <c r="D85" s="11" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="E85" s="11">
         <v>1</v>
@@ -4528,16 +4785,16 @@
     </row>
     <row r="86" spans="1:11" ht="28.8">
       <c r="A86" s="9" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B86" s="9" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C86" s="10">
         <v>13091001</v>
       </c>
       <c r="D86" s="11" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="E86" s="11">
         <v>1</v>
@@ -4559,13 +4816,13 @@
     </row>
     <row r="87" spans="1:11">
       <c r="A87" s="9" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="B87" s="9" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="C87" s="10" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="D87" s="11" t="s">
         <v>51</v>
@@ -4591,10 +4848,10 @@
     <row r="88" spans="1:11" ht="28.8">
       <c r="A88" s="9"/>
       <c r="B88" s="9" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C88" s="10" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="D88" s="11" t="s">
         <v>51</v>
@@ -4609,7 +4866,7 @@
         <v>17</v>
       </c>
       <c r="H88" s="9" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="I88" s="11">
         <v>16</v>
@@ -4621,13 +4878,13 @@
     </row>
     <row r="89" spans="1:11" ht="28.8">
       <c r="A89" s="9" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="B89" s="9" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="C89" s="10" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="D89" s="11" t="s">
         <v>51</v>
@@ -4652,13 +4909,13 @@
     </row>
     <row r="90" spans="1:11" ht="43.2">
       <c r="A90" s="9" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="B90" s="9" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C90" s="10" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="D90" s="11" t="s">
         <v>51</v>
@@ -4683,13 +4940,13 @@
     </row>
     <row r="91" spans="1:11" ht="28.8">
       <c r="A91" s="9" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="B91" s="9" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C91" s="10" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="D91" s="11" t="s">
         <v>51</v>
@@ -4714,13 +4971,13 @@
     </row>
     <row r="92" spans="1:11" ht="28.8">
       <c r="A92" s="9" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="B92" s="9" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C92" s="10" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="D92" s="11" t="s">
         <v>51</v>
@@ -4745,13 +5002,13 @@
     </row>
     <row r="93" spans="1:11" ht="28.8">
       <c r="A93" s="9" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="B93" s="9" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="C93" s="10" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="D93" s="11" t="s">
         <v>51</v>
@@ -4776,13 +5033,13 @@
     </row>
     <row r="94" spans="1:11" ht="28.8">
       <c r="A94" s="9" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="B94" s="9" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C94" s="10" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="D94" s="11" t="s">
         <v>51</v>
@@ -4807,13 +5064,13 @@
     </row>
     <row r="95" spans="1:11" ht="28.8">
       <c r="A95" s="9" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="B95" s="9" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="C95" s="10" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="D95" s="11" t="s">
         <v>51</v>
@@ -4822,7 +5079,7 @@
       <c r="F95" s="9"/>
       <c r="G95" s="11"/>
       <c r="H95" s="9" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="I95" s="11">
         <v>2</v>
@@ -4832,18 +5089,18 @@
         <v>-2</v>
       </c>
       <c r="K95" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
     </row>
     <row r="96" spans="1:11" ht="28.8">
       <c r="A96" s="9" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="B96" s="9" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="C96" s="10" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="D96" s="11" t="s">
         <v>51</v>
@@ -4869,10 +5126,10 @@
     <row r="97" spans="1:11" ht="28.8">
       <c r="A97" s="9"/>
       <c r="B97" s="9" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="C97" s="10" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="D97" s="11" t="s">
         <v>51</v>
@@ -4887,7 +5144,7 @@
         <v>17</v>
       </c>
       <c r="H97" s="9" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="I97" s="11">
         <v>6</v>
@@ -4899,13 +5156,13 @@
     </row>
     <row r="98" spans="1:11" ht="28.8">
       <c r="A98" s="9" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="B98" s="9" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="C98" s="10" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="D98" s="11" t="s">
         <v>51</v>
@@ -4930,13 +5187,13 @@
     </row>
     <row r="99" spans="1:11" ht="28.8">
       <c r="A99" s="9" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="B99" s="9" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="C99" s="10" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="D99" s="11" t="s">
         <v>51</v>
@@ -4955,16 +5212,16 @@
         <v>2</v>
       </c>
       <c r="J99" s="7">
-        <f t="shared" ref="J99:J114" si="3">IF(ISBLANK(I99),"",E99-I99)</f>
+        <f t="shared" ref="J99:J113" si="3">IF(ISBLANK(I99),"",E99-I99)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:11" ht="28.8">
+    <row r="100" spans="1:11" ht="47.4" customHeight="1">
       <c r="A100" s="9" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="B100" s="9" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="C100" s="10">
         <v>29450</v>
@@ -4981,30 +5238,28 @@
       <c r="G100" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H100" s="9" t="s">
-        <v>188</v>
-      </c>
+      <c r="H100" s="9"/>
       <c r="I100" s="11"/>
       <c r="J100" s="7" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K100" s="19" t="s">
-        <v>326</v>
+      <c r="K100" s="28" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="101" spans="1:11">
       <c r="A101" s="9" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="B101" s="9" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C101" s="10" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="D101" s="11" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="E101" s="11">
         <v>2</v>
@@ -5027,13 +5282,13 @@
     <row r="102" spans="1:11">
       <c r="A102" s="9"/>
       <c r="B102" s="9" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="C102" s="10" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="D102" s="11" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="E102" s="11">
         <v>1</v>
@@ -5050,154 +5305,156 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K102" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="103" spans="1:11" ht="43.2">
+      <c r="K102" s="31" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" ht="60" customHeight="1">
       <c r="A103" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="B103" s="33" t="s">
+        <v>241</v>
+      </c>
+      <c r="C103" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="D103" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="E103" s="11">
+        <v>1</v>
+      </c>
+      <c r="F103" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G103" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H103" s="9"/>
+      <c r="I103" s="11">
+        <v>1</v>
+      </c>
+      <c r="J103" s="7">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="K103" s="19"/>
+    </row>
+    <row r="104" spans="1:11" ht="28.8">
+      <c r="A104" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="B104" s="9" t="s">
         <v>245</v>
       </c>
-      <c r="B103" s="22" t="s">
+      <c r="C104" s="10">
+        <v>2864011</v>
+      </c>
+      <c r="D104" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="E104" s="11">
+        <v>2</v>
+      </c>
+      <c r="F104" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G104" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H104" s="9"/>
+      <c r="I104" s="11">
+        <v>2</v>
+      </c>
+      <c r="J104" s="7">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" ht="28.8">
+      <c r="A105" s="9" t="s">
         <v>246</v>
       </c>
-      <c r="C103" s="10" t="s">
+      <c r="B105" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="D103" s="11" t="s">
+      <c r="C105" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="E103" s="11">
-        <v>1</v>
-      </c>
-      <c r="F103" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G103" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="H103" s="15" t="s">
+      <c r="D105" s="11" t="s">
         <v>249</v>
       </c>
-      <c r="I103" s="11"/>
-      <c r="J103" s="7" t="str">
+      <c r="E105" s="11">
+        <v>2</v>
+      </c>
+      <c r="F105" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G105" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="H105" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="I105" s="11"/>
+      <c r="J105" s="7" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K103" s="19" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="104" spans="1:11" ht="43.2">
-      <c r="A104" s="9" t="s">
-        <v>250</v>
-      </c>
-      <c r="B104" s="9" t="s">
+      <c r="K105" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" ht="72">
+      <c r="A106" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="C104" s="10" t="s">
-        <v>247</v>
-      </c>
-      <c r="D104" s="11" t="s">
-        <v>248</v>
-      </c>
-      <c r="E104" s="11"/>
-      <c r="F104" s="11"/>
-      <c r="G104" s="11"/>
-      <c r="H104" s="9" t="s">
+      <c r="B106" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="I104" s="11">
-        <v>1</v>
-      </c>
-      <c r="J104" s="7">
-        <f t="shared" si="3"/>
-        <v>-1</v>
-      </c>
-      <c r="K104" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="105" spans="1:11" ht="28.8">
-      <c r="A105" s="9" t="s">
+      <c r="C106" s="10" t="s">
         <v>253</v>
       </c>
-      <c r="B105" s="9" t="s">
+      <c r="D106" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="E106" s="11">
+        <v>5</v>
+      </c>
+      <c r="F106" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G106" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H106" s="15" t="s">
         <v>254</v>
-      </c>
-      <c r="C105" s="10">
-        <v>2864011</v>
-      </c>
-      <c r="D105" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="E105" s="11">
-        <v>2</v>
-      </c>
-      <c r="F105" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G105" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="H105" s="9"/>
-      <c r="I105" s="11">
-        <v>2</v>
-      </c>
-      <c r="J105" s="7">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106" spans="1:11" ht="28.8">
-      <c r="A106" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="B106" s="9" t="s">
-        <v>256</v>
-      </c>
-      <c r="C106" s="10" t="s">
-        <v>257</v>
-      </c>
-      <c r="D106" s="11" t="s">
-        <v>258</v>
-      </c>
-      <c r="E106" s="11">
-        <v>2</v>
-      </c>
-      <c r="F106" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G106" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="H106" s="9" t="s">
-        <v>259</v>
       </c>
       <c r="I106" s="11"/>
       <c r="J106" s="7" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K106" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="107" spans="1:11" ht="86.4">
+      <c r="K106" s="34" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" ht="43.2">
       <c r="A107" s="9" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="B107" s="9" t="s">
-        <v>261</v>
-      </c>
-      <c r="C107" s="10" t="s">
-        <v>262</v>
+        <v>256</v>
+      </c>
+      <c r="C107" s="22" t="s">
+        <v>320</v>
       </c>
       <c r="D107" s="11" t="s">
         <v>116</v>
       </c>
       <c r="E107" s="11">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="F107" s="11" t="s">
         <v>19</v>
@@ -5205,27 +5462,26 @@
       <c r="G107" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="H107" s="15" t="s">
-        <v>263</v>
-      </c>
-      <c r="I107" s="11"/>
-      <c r="J107" s="7" t="str">
+      <c r="H107" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="I107" s="11">
+        <v>9</v>
+      </c>
+      <c r="J107" s="7">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K107" s="1" t="s">
-        <v>331</v>
+        <v>4</v>
       </c>
     </row>
     <row r="108" spans="1:11" ht="43.2">
       <c r="A108" s="9" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="B108" s="9" t="s">
-        <v>265</v>
-      </c>
-      <c r="C108" s="23" t="s">
-        <v>332</v>
+        <v>258</v>
+      </c>
+      <c r="C108" s="10" t="s">
+        <v>259</v>
       </c>
       <c r="D108" s="11" t="s">
         <v>116</v>
@@ -5240,7 +5496,7 @@
         <v>17</v>
       </c>
       <c r="H108" s="9" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="I108" s="11">
         <v>9</v>
@@ -5250,21 +5506,21 @@
         <v>4</v>
       </c>
     </row>
-    <row r="109" spans="1:11" ht="43.2">
+    <row r="109" spans="1:11" ht="28.8">
       <c r="A109" s="9" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="B109" s="9" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="C109" s="10" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="D109" s="11" t="s">
         <v>116</v>
       </c>
       <c r="E109" s="11">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F109" s="11" t="s">
         <v>19</v>
@@ -5272,32 +5528,33 @@
       <c r="G109" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="H109" s="9" t="s">
-        <v>266</v>
-      </c>
-      <c r="I109" s="11">
-        <v>9</v>
-      </c>
-      <c r="J109" s="7">
+      <c r="H109" s="18" t="s">
+        <v>263</v>
+      </c>
+      <c r="I109" s="11"/>
+      <c r="J109" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v/>
+      </c>
+      <c r="K109" s="29" t="s">
+        <v>321</v>
       </c>
     </row>
     <row r="110" spans="1:11" ht="28.8">
       <c r="A110" s="9" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="B110" s="9" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C110" s="10" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="D110" s="11" t="s">
         <v>116</v>
       </c>
       <c r="E110" s="11">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F110" s="11" t="s">
         <v>19</v>
@@ -5306,98 +5563,100 @@
         <v>17</v>
       </c>
       <c r="H110" s="18" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="I110" s="11"/>
       <c r="J110" s="7" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K110" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="111" spans="1:11" ht="28.8">
+      <c r="K110" s="34" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" ht="43.2">
       <c r="A111" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="B111" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="C111" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="D111" s="11" t="s">
+        <v>270</v>
+      </c>
+      <c r="E111" s="11">
+        <v>1</v>
+      </c>
+      <c r="F111" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G111" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H111" s="9"/>
+      <c r="I111" s="11">
+        <v>1</v>
+      </c>
+      <c r="J111" s="7">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="K111" s="1"/>
+    </row>
+    <row r="112" spans="1:11" ht="57.6">
+      <c r="A112" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="B112" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="C112" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="D112" s="11" t="s">
+        <v>270</v>
+      </c>
+      <c r="E112" s="11">
+        <v>5</v>
+      </c>
+      <c r="F112" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G112" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H112" s="9" t="s">
         <v>273</v>
       </c>
-      <c r="B111" s="9" t="s">
-        <v>274</v>
-      </c>
-      <c r="C111" s="10" t="s">
-        <v>275</v>
-      </c>
-      <c r="D111" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="E111" s="11">
-        <v>3</v>
-      </c>
-      <c r="F111" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G111" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H111" s="18" t="s">
-        <v>272</v>
-      </c>
-      <c r="I111" s="11"/>
-      <c r="J111" s="7" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K111" s="1" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="112" spans="1:11" ht="43.2">
-      <c r="A112" s="9" t="s">
-        <v>276</v>
-      </c>
-      <c r="B112" s="9" t="s">
-        <v>277</v>
-      </c>
-      <c r="C112" s="10" t="s">
-        <v>278</v>
-      </c>
-      <c r="D112" s="11" t="s">
-        <v>279</v>
-      </c>
-      <c r="E112" s="11">
-        <v>1</v>
-      </c>
-      <c r="F112" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G112" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="H112" s="9"/>
       <c r="I112" s="11">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J112" s="7">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K112" s="1"/>
-    </row>
-    <row r="113" spans="1:11" ht="57.6">
+        <v>-2</v>
+      </c>
+      <c r="K112" s="35" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" ht="72">
       <c r="A113" s="9" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="B113" s="9" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="C113" s="10" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="D113" s="11" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="E113" s="11">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F113" s="11" t="s">
         <v>19</v>
@@ -5405,70 +5664,63 @@
       <c r="G113" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H113" s="9" t="s">
-        <v>283</v>
-      </c>
+      <c r="H113" s="9"/>
       <c r="I113" s="11">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J113" s="7">
         <f t="shared" si="3"/>
-        <v>-2</v>
-      </c>
-      <c r="K113" s="24" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="114" spans="1:11" ht="72">
-      <c r="A114" s="9" t="s">
-        <v>284</v>
-      </c>
-      <c r="B114" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="C114" s="10" t="s">
-        <v>286</v>
-      </c>
-      <c r="D114" s="11" t="s">
-        <v>279</v>
-      </c>
-      <c r="E114" s="11">
-        <v>2</v>
-      </c>
-      <c r="F114" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G114" s="11" t="s">
-        <v>17</v>
-      </c>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10">
+      <c r="A114" s="9"/>
+      <c r="B114" s="9"/>
+      <c r="C114" s="10"/>
+      <c r="D114" s="11"/>
+      <c r="E114" s="11"/>
+      <c r="F114" s="11"/>
+      <c r="G114" s="11"/>
       <c r="H114" s="9"/>
-      <c r="I114" s="11">
-        <v>2</v>
-      </c>
-      <c r="J114" s="7">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="115" spans="1:11">
+      <c r="I114" s="11"/>
+      <c r="J114" s="7"/>
+    </row>
+    <row r="115" spans="1:10" ht="43.2">
       <c r="A115" s="9"/>
-      <c r="B115" s="9"/>
-      <c r="C115" s="10"/>
-      <c r="D115" s="11"/>
-      <c r="E115" s="11"/>
-      <c r="F115" s="11"/>
-      <c r="G115" s="11"/>
+      <c r="B115" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="C115" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="D115" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E115" s="11">
+        <v>1</v>
+      </c>
+      <c r="F115" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G115" s="11" t="s">
+        <v>17</v>
+      </c>
       <c r="H115" s="9"/>
       <c r="I115" s="11"/>
-      <c r="J115" s="7"/>
-    </row>
-    <row r="116" spans="1:11" ht="43.2">
-      <c r="A116" s="9"/>
+      <c r="J115" s="7" t="str">
+        <f t="shared" ref="J115:J122" si="4">IF(ISBLANK(I115),"",E115-I115)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116" spans="1:10" ht="28.8">
+      <c r="A116" s="9" t="s">
+        <v>279</v>
+      </c>
       <c r="B116" s="9" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="C116" s="10" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="D116" s="11" t="s">
         <v>15</v>
@@ -5485,28 +5737,26 @@
       <c r="H116" s="9"/>
       <c r="I116" s="11"/>
       <c r="J116" s="7" t="str">
-        <f t="shared" ref="J116:J123" si="4">IF(ISBLANK(I116),"",E116-I116)</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
-    <row r="117" spans="1:11" ht="28.8">
-      <c r="A117" s="9" t="s">
-        <v>289</v>
-      </c>
+    <row r="117" spans="1:10" ht="28.8">
+      <c r="A117" s="9"/>
       <c r="B117" s="9" t="s">
-        <v>290</v>
-      </c>
-      <c r="C117" s="10" t="s">
-        <v>291</v>
+        <v>124</v>
+      </c>
+      <c r="C117" s="10">
+        <v>1020100000</v>
       </c>
       <c r="D117" s="11" t="s">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="E117" s="11">
         <v>1</v>
       </c>
       <c r="F117" s="11" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G117" s="11" t="s">
         <v>17</v>
@@ -5518,42 +5768,46 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="1:11" ht="28.8">
-      <c r="A118" s="9"/>
+    <row r="118" spans="1:10">
+      <c r="A118" s="9" t="s">
+        <v>282</v>
+      </c>
       <c r="B118" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="C118" s="10">
-        <v>1020100000</v>
+        <v>283</v>
+      </c>
+      <c r="C118" s="14" t="s">
+        <v>284</v>
       </c>
       <c r="D118" s="11" t="s">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="E118" s="11">
         <v>1</v>
       </c>
       <c r="F118" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="G118" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="H118" s="9"/>
+        <v>19</v>
+      </c>
+      <c r="G118" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="H118" s="9" t="s">
+        <v>285</v>
+      </c>
       <c r="I118" s="11"/>
       <c r="J118" s="7" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
-    <row r="119" spans="1:11">
+    <row r="119" spans="1:10">
       <c r="A119" s="9" t="s">
-        <v>292</v>
+        <v>37</v>
       </c>
       <c r="B119" s="9" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="C119" s="14" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="D119" s="11" t="s">
         <v>15</v>
@@ -5568,7 +5822,7 @@
         <v>103</v>
       </c>
       <c r="H119" s="9" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="I119" s="11"/>
       <c r="J119" s="7" t="str">
@@ -5576,15 +5830,15 @@
         <v/>
       </c>
     </row>
-    <row r="120" spans="1:11">
+    <row r="120" spans="1:10">
       <c r="A120" s="9" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="B120" s="9" t="s">
-        <v>296</v>
-      </c>
-      <c r="C120" s="14" t="s">
-        <v>297</v>
+        <v>288</v>
+      </c>
+      <c r="C120" s="10" t="s">
+        <v>289</v>
       </c>
       <c r="D120" s="11" t="s">
         <v>15</v>
@@ -5599,7 +5853,7 @@
         <v>103</v>
       </c>
       <c r="H120" s="9" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="I120" s="11"/>
       <c r="J120" s="7" t="str">
@@ -5607,15 +5861,15 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="1:11">
+    <row r="121" spans="1:10">
       <c r="A121" s="9" t="s">
-        <v>46</v>
+        <v>290</v>
       </c>
       <c r="B121" s="9" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="C121" s="10" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="D121" s="11" t="s">
         <v>15</v>
@@ -5630,7 +5884,7 @@
         <v>103</v>
       </c>
       <c r="H121" s="9" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="I121" s="11"/>
       <c r="J121" s="7" t="str">
@@ -5638,15 +5892,15 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="1:11">
+    <row r="122" spans="1:10">
       <c r="A122" s="9" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="B122" s="9" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="C122" s="10" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="D122" s="11" t="s">
         <v>15</v>
@@ -5661,7 +5915,7 @@
         <v>103</v>
       </c>
       <c r="H122" s="9" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="I122" s="11"/>
       <c r="J122" s="7" t="str">
@@ -5669,114 +5923,109 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="1:11">
-      <c r="A123" s="9" t="s">
-        <v>303</v>
-      </c>
-      <c r="B123" s="9" t="s">
-        <v>304</v>
-      </c>
-      <c r="C123" s="10" t="s">
-        <v>305</v>
-      </c>
-      <c r="D123" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="E123" s="11">
-        <v>1</v>
-      </c>
-      <c r="F123" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G123" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="H123" s="9" t="s">
-        <v>295</v>
-      </c>
-      <c r="I123" s="11"/>
-      <c r="J123" s="7" t="str">
-        <f t="shared" si="4"/>
+    <row r="123" spans="1:10">
+      <c r="A123" s="9"/>
+      <c r="B123" s="9"/>
+      <c r="C123" s="10"/>
+      <c r="D123" s="11"/>
+      <c r="E123" s="11"/>
+      <c r="F123" s="11"/>
+      <c r="G123" s="11"/>
+      <c r="H123" s="9"/>
+      <c r="I123" s="17"/>
+      <c r="J123" s="7"/>
+    </row>
+    <row r="124" spans="1:10" ht="226.95" customHeight="1">
+      <c r="A124" s="24"/>
+      <c r="B124" s="26" t="s">
+        <v>296</v>
+      </c>
+      <c r="C124" s="25" t="s">
+        <v>297</v>
+      </c>
+      <c r="D124" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="E124" s="27">
+        <v>1</v>
+      </c>
+      <c r="F124" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="G124" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="H124" s="24"/>
+      <c r="I124" s="24"/>
+      <c r="J124" s="25" t="str">
+        <f>IF(ISBLANK(I124), "", E124-I124)</f>
         <v/>
       </c>
     </row>
-    <row r="124" spans="1:11">
-      <c r="A124" s="9"/>
-      <c r="B124" s="9"/>
-      <c r="C124" s="10"/>
-      <c r="D124" s="11"/>
-      <c r="E124" s="11"/>
-      <c r="F124" s="11"/>
-      <c r="G124" s="11"/>
-      <c r="H124" s="9"/>
-      <c r="I124" s="17"/>
-      <c r="J124" s="7"/>
-    </row>
-    <row r="125" spans="1:11" ht="226.95" customHeight="1">
-      <c r="A125" s="26"/>
-      <c r="B125" s="28" t="s">
-        <v>306</v>
-      </c>
-      <c r="C125" s="27" t="s">
-        <v>307</v>
-      </c>
-      <c r="D125" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="E125" s="29">
-        <v>1</v>
-      </c>
-      <c r="F125" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="G125" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="H125" s="26"/>
-      <c r="I125" s="26"/>
-      <c r="J125" s="27" t="str">
-        <f>IF(ISBLANK(I125), "", E125-I125)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="126" spans="1:11" ht="226.95" customHeight="1">
-      <c r="A126" s="26"/>
-      <c r="B126" s="28"/>
-      <c r="C126" s="27"/>
-      <c r="D126" s="25"/>
-      <c r="E126" s="29"/>
-      <c r="F126" s="25"/>
-      <c r="G126" s="25"/>
-      <c r="H126" s="26"/>
-      <c r="I126" s="26"/>
-      <c r="J126" s="27"/>
+    <row r="125" spans="1:10" ht="226.95" customHeight="1">
+      <c r="A125" s="24"/>
+      <c r="B125" s="26"/>
+      <c r="C125" s="25"/>
+      <c r="D125" s="23"/>
+      <c r="E125" s="27"/>
+      <c r="F125" s="23"/>
+      <c r="G125" s="23"/>
+      <c r="H125" s="24"/>
+      <c r="I125" s="24"/>
+      <c r="J125" s="25"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:F116" xr:uid="{22550ED4-55A0-4F53-98B1-D10F42FD3934}"/>
+  <autoFilter ref="B1:F115" xr:uid="{22550ED4-55A0-4F53-98B1-D10F42FD3934}"/>
   <mergeCells count="10">
-    <mergeCell ref="G125:G126"/>
-    <mergeCell ref="H125:H126"/>
-    <mergeCell ref="I125:I126"/>
-    <mergeCell ref="J125:J126"/>
-    <mergeCell ref="A125:A126"/>
-    <mergeCell ref="B125:B126"/>
-    <mergeCell ref="C125:C126"/>
-    <mergeCell ref="D125:D126"/>
-    <mergeCell ref="E125:E126"/>
-    <mergeCell ref="F125:F126"/>
+    <mergeCell ref="G124:G125"/>
+    <mergeCell ref="H124:H125"/>
+    <mergeCell ref="I124:I125"/>
+    <mergeCell ref="J124:J125"/>
+    <mergeCell ref="A124:A125"/>
+    <mergeCell ref="B124:B125"/>
+    <mergeCell ref="C124:C125"/>
+    <mergeCell ref="D124:D125"/>
+    <mergeCell ref="E124:E125"/>
+    <mergeCell ref="F124:F125"/>
   </mergeCells>
-  <conditionalFormatting sqref="J1:J33 J35:J125 J127:J1048576">
+  <conditionalFormatting sqref="J1:J33 J126:J1048576 J35:J124">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75" bottom="0.75" header="0.30000000000000004" footer="0.30000000000000004"/>
-  <pageSetup paperSize="0" fitToWidth="0" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="v">
-      <legacyDrawing r:id="rId2"/>
+      <legacyDrawing r:id="rId3"/>
     </mc:Choice>
   </mc:AlternateContent>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA14BE4E-0550-4764-9E84-993432B630D6}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>328</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>